<commit_message>
chore: regenerate xlsx test data to match CSV
Disbursed statuses blanked (blank defaults to Disbursed); only the On Hold
term is labelled. Built from the CSV text directly so contact numbers keep
their leading zero.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scholar_migration_test_data.xlsx
+++ b/scholar_migration_test_data.xlsx
@@ -676,7 +676,7 @@
         <v>25000</v>
       </c>
       <c r="V2" t="str">
-        <v>Disbursed</v>
+        <v/>
       </c>
       <c r="W2" t="str">
         <v/>
@@ -834,7 +834,7 @@
         <v>25000</v>
       </c>
       <c r="V3" t="str">
-        <v>Disbursed</v>
+        <v/>
       </c>
       <c r="W3" t="str">
         <v>2024-2025</v>
@@ -849,7 +849,7 @@
         <v>25000</v>
       </c>
       <c r="AA3" t="str">
-        <v>Disbursed</v>
+        <v/>
       </c>
       <c r="AB3" t="str">
         <v>2025-2026</v>
@@ -864,7 +864,7 @@
         <v>25000</v>
       </c>
       <c r="AF3" t="str">
-        <v>Disbursed</v>
+        <v/>
       </c>
       <c r="AG3" t="str">
         <v/>
@@ -992,7 +992,7 @@
         <v>25000</v>
       </c>
       <c r="V4" t="str">
-        <v>Disbursed</v>
+        <v/>
       </c>
       <c r="W4" t="str">
         <v>2023-2024</v>
@@ -1007,7 +1007,7 @@
         <v>25000</v>
       </c>
       <c r="AA4" t="str">
-        <v>Disbursed</v>
+        <v/>
       </c>
       <c r="AB4" t="str">
         <v>2024-2025</v>
@@ -1037,7 +1037,7 @@
         <v>25000</v>
       </c>
       <c r="AK4" t="str">
-        <v>Disbursed</v>
+        <v/>
       </c>
       <c r="AL4" t="str">
         <v>2025-2026</v>
@@ -1052,7 +1052,7 @@
         <v>25000</v>
       </c>
       <c r="AP4" t="str">
-        <v>Disbursed</v>
+        <v/>
       </c>
       <c r="AQ4" t="str">
         <v/>
@@ -1150,7 +1150,7 @@
         <v>25000</v>
       </c>
       <c r="V5" t="str">
-        <v>Disbursed</v>
+        <v/>
       </c>
       <c r="W5" t="str">
         <v>2022-2023</v>
@@ -1165,7 +1165,7 @@
         <v>25000</v>
       </c>
       <c r="AA5" t="str">
-        <v>Disbursed</v>
+        <v/>
       </c>
       <c r="AB5" t="str">
         <v>2023-2024</v>
@@ -1180,7 +1180,7 @@
         <v>25000</v>
       </c>
       <c r="AF5" t="str">
-        <v>Disbursed</v>
+        <v/>
       </c>
       <c r="AG5" t="str">
         <v>2023-2024</v>
@@ -1195,7 +1195,7 @@
         <v>25000</v>
       </c>
       <c r="AK5" t="str">
-        <v>Disbursed</v>
+        <v/>
       </c>
       <c r="AL5" t="str">
         <v>2024-2025</v>
@@ -1210,7 +1210,7 @@
         <v>25000</v>
       </c>
       <c r="AP5" t="str">
-        <v>Disbursed</v>
+        <v/>
       </c>
       <c r="AQ5" t="str">
         <v>2024-2025</v>
@@ -1225,7 +1225,7 @@
         <v>25000</v>
       </c>
       <c r="AU5" t="str">
-        <v>Disbursed</v>
+        <v/>
       </c>
       <c r="AV5" t="str">
         <v>2025-2026</v>
@@ -1240,7 +1240,7 @@
         <v>25000</v>
       </c>
       <c r="AZ5" t="str">
-        <v>Disbursed</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>